<commit_message>
Ajuste de referencia a nombre del fichero
</commit_message>
<xml_diff>
--- a/datos/raw/Fuentes oficiales de los ficheros.xlsx
+++ b/datos/raw/Fuentes oficiales de los ficheros.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Education\Master BigData IA\TFM\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Education\Master BigData IA\TFM\Proyecto prediccion electoral\tfm-electoral-colombia\datos\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA136C12-1017-496B-9281-2475C8993E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771C0957-1341-4108-B9B0-6DC1FDAC3CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-1230" windowWidth="29040" windowHeight="15720" xr2:uid="{48246D06-CF5A-496A-9332-3BB18996AF97}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{48246D06-CF5A-496A-9332-3BB18996AF97}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -75,9 +75,6 @@
     <t>anexo_dptal_pobreza_multidimensional_2022.xlsx</t>
   </si>
   <si>
-    <t>VICTIMAS_FILTRADO.csv</t>
-  </si>
-  <si>
     <t>MMV_NACIONAL_PRESIDENTE_2022_1v.csv</t>
   </si>
   <si>
@@ -130,6 +127,9 @@
   </si>
   <si>
     <t>IPM</t>
+  </si>
+  <si>
+    <t>VICTIMAS_FILTRADO_V2.csv</t>
   </si>
 </sst>
 </file>
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -347,10 +347,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -679,124 +678,125 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="1.21875" customWidth="1"/>
-    <col min="2" max="3" width="49" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="3" max="3" width="49" customWidth="1"/>
     <col min="4" max="4" width="118.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="6.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:4" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="15"/>
+      <c r="B3" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="7"/>
-      <c r="C5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="9"/>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="8"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="7"/>
-      <c r="C6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="9"/>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="8"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
-      <c r="C7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="9"/>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="7"/>
-      <c r="C8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="9"/>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="8"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="7"/>
-      <c r="C9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="9"/>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="8"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="7"/>
-      <c r="C10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="9"/>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="8"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="7"/>
-      <c r="C11" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="9"/>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="8"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12" s="7"/>
-      <c r="C12" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="9"/>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="8"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B13" s="7"/>
-      <c r="C13" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="9"/>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="8"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B14" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="15"/>
+      <c r="C15" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="16"/>
-      <c r="C15" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="18"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="2:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="6"/>
@@ -805,57 +805,57 @@
       <c r="B17" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="15"/>
+      <c r="B18" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="14"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B19" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="17" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="6"/>
     </row>
     <row r="22" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="11" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>